<commit_message>
Modified Systems Report with totals, and only displays the active variant component
</commit_message>
<xml_diff>
--- a/data/input_tables/Properties.xlsx
+++ b/data/input_tables/Properties.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kkoch28\Downloads\NAVSEA RESEARCH\data\input_tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF69EFD-376C-45F3-9291-445E25CA3565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C7BD9F7-4D26-4ABA-BC96-72C0BA7B55BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1388" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1390" uniqueCount="106">
   <si>
     <t>Profile--&gt;</t>
   </si>
@@ -1704,11 +1704,11 @@
       <c r="H8" t="b">
         <v>1</v>
       </c>
-      <c r="I8">
-        <v>151</v>
-      </c>
-      <c r="J8" t="b">
-        <v>1</v>
+      <c r="I8" t="s">
+        <v>61</v>
+      </c>
+      <c r="J8" t="s">
+        <v>61</v>
       </c>
       <c r="K8">
         <v>7.0000000000000001E-3</v>

</xml_diff>